<commit_message>
Prepare llm_values_2026_06 handoff package
</commit_message>
<xml_diff>
--- a/results/analysis/stage0_vs_stage3/english_advantage_average.xlsx
+++ b/results/analysis/stage0_vs_stage3/english_advantage_average.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,6 +441,26 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>native_distance</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>english_distance</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>cultural_region</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>is_islamic</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>english_advantage</t>
         </is>
       </c>
@@ -448,46 +468,88 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zh-hk</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>47.96754218421044</v>
+        <v>2.152718260122653</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.565473554732652</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>27.27921792034887</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Taiwan, Province of China</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>zh-cn</t>
+          <t>zh-tw</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>25.20136153734433</v>
+        <v>2.732502794981023</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.993229331105257</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>27.05481089474604</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.43205357549388</v>
+        <v>1.441361964730207</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.077500970564295</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>25.24424836158482</v>
       </c>
     </row>
     <row r="5">
@@ -498,32 +560,60 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>zh-cn</t>
+          <t>zh-hk</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13.01537760899442</v>
+        <v>2.073007698556737</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.559300736505874</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>24.78075515148906</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Taiwan (Province of China)</t>
+          <t>Palestine</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zh-tw</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>12.44300409936053</v>
+        <v>2.186651604619046</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.657829276397343</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>24.18411452032996</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -532,133 +622,259 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.00074404313217</v>
+        <v>2.556536807966632</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.022455649350871</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>20.89080653763589</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5.055780452533421</v>
+        <v>3.279106960538209</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.610802580271304</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20.38068255502146</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>es</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3.24397347402226</v>
+        <v>1.639568852538827</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.314534461207084</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>19.82438192994678</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.289142725553169</v>
+        <v>1.873601855201179</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.536178583017985</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>18.00933700222894</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Korea (the Republic of)</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ko</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.1349453795457762</v>
+        <v>2.696641982259508</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.220567128480993</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>17.65435889934538</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Mali</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ar</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.8732210730049044</v>
+        <v>2.430885855219917</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.003648613331353</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>17.57537240883375</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-1.087060315157804</v>
+        <v>3.623121046583009</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.987164180452518</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>17.55273583062499</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Burkina Faso</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>fr</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-2.641947633166856</v>
+        <v>2.144361283781751</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.768958116882958</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>17.50652605687507</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Macao</t>
+          <t>Nicaragua</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>zh-cn</t>
+          <t>es</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-3.276537414548494</v>
+        <v>1.917945616259785</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.584885519531082</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>17.365460934091</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -667,133 +883,259 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-4.484200899408044</v>
+        <v>2.557756251373463</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.126295819507233</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16.86870794019344</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-6.599422185524415</v>
+        <v>2.100353952992315</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.764340156173555</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>15.99796055041344</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ar</t>
+          <t>zh-cn</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-7.251724257936232</v>
+        <v>1.85279039983711</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.559300736505874</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F18" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>15.84041364619758</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-9.081914149368167</v>
+        <v>1.874864569666324</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.593035688469196</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>15.03195941492914</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>zh-cn</t>
+          <t>es</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-13.51502250514504</v>
+        <v>2.182928199424994</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1.895263565665109</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>13.17792467180821</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ar</t>
+          <t>es</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-17.22456013349373</v>
+        <v>1.792419402070336</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.576793639313436</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F21" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>12.02987216651647</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Taiwan (Province of China)</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>zh-cn</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-22.73223590979841</v>
+        <v>1.918572100358398</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.710878702268348</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>10.82541532065705</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>es</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-23.58352449497422</v>
+        <v>2.227043906818228</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.995443080666642</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F23" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>10.3994728367288</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Russian Federation (the)</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ru</t>
+          <t>es</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-25.03902508059246</v>
+        <v>1.879703281541393</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.699508452883641</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>9.586344314406297</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -802,112 +1144,804 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-26.25404308017669</v>
+        <v>2.140874153914743</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2.011616772193522</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6.037598309310464</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>ru</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>-35.58549122363982</v>
+        <v>1.292860430109726</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1.228741731853664</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4.95944471365867</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Macao</t>
+          <t>Libya</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>zh-hk</t>
+          <t>ar</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>-39.42548368917618</v>
+        <v>2.294036001257761</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2.189799191472093</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>African-Islamic</t>
+        </is>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4.543817521979484</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>pt</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>-40.41285854258323</v>
+        <v>2.019670016789068</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.947410079463477</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>3.577809083905269</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>-50.56781025673673</v>
+        <v>1.849014387958417</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.787684277706038</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F29" t="b">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3.316908221579431</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>es</t>
+          <t>ko</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-52.26705337580289</v>
+        <v>1.497567019785533</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.453122962123065</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2.967750830198766</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ar</t>
+          <t>ru</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>-54.47703008645142</v>
+        <v>1.477156617151254</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.449529059700356</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>West &amp; South Asia</t>
+        </is>
+      </c>
+      <c r="F31" t="b">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1.870320122464661</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Macao</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1.505472760569258</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1.478039842226193</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1.82221286638836</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>zh-cn</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.9744281780600765</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.9737133587944449</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.07335781966555469</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Belarus</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1.532085672515696</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.546248865064457</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Orthodox Europe</t>
+        </is>
+      </c>
+      <c r="F34" t="b">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-0.9244386787786055</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1.357502077555349</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1.387946302992809</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F35" t="b">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-2.242665108276269</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2.350011823873006</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2.412889974983115</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F36" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-2.675652542312811</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1.948532799983175</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2.001471510584124</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F37" t="b">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-2.716849857564957</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3.048175886555469</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3.204411326824733</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F38" t="b">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-5.125538882397468</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2.770045992833987</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2.973740008338852</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F39" t="b">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-7.353452470890877</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2.149981129497089</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2.31650090177838</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Protestant Europe</t>
+        </is>
+      </c>
+      <c r="F40" t="b">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-7.745173666721588</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Venezuela</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.759658136978508</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3.03358859615972</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-9.926246135730871</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1.699867864407737</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.900672216589812</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F42" t="b">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-11.81293889875601</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>es</t>
         </is>
       </c>
-      <c r="C32" t="n">
-        <v>-87.18824285956654</v>
+      <c r="C43" t="n">
+        <v>2.205486633109636</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.472562238252999</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F43" t="b">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-12.10959981048709</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2.340864544152464</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2.65210390261424</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F44" t="b">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-13.29591493191092</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Macao</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>zh-cn</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.30150555812365</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.478039842226193</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Confucian</t>
+        </is>
+      </c>
+      <c r="F45" t="b">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-13.56385172546238</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2.032425450963471</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2.31650090177838</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Protestant Europe</t>
+        </is>
+      </c>
+      <c r="F46" t="b">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-13.97716460794383</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.48999710248082</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.869280568255204</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F47" t="b">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-15.23228542701909</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2.358292143366335</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.869280568255204</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F48" t="b">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-21.66773214786951</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2.419658269871729</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2.973740008338852</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F49" t="b">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-22.89917321657554</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1.427123268153301</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1.776729956178061</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Catholic Europe</t>
+        </is>
+      </c>
+      <c r="F50" t="b">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-24.49730137727712</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1.848535341291206</v>
+      </c>
+      <c r="D51" t="n">
+        <v>2.331509659898773</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Protestant Europe</t>
+        </is>
+      </c>
+      <c r="F51" t="b">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-26.12740518502653</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1.735072984987228</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2.31650090177838</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Protestant Europe</t>
+        </is>
+      </c>
+      <c r="F52" t="b">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-33.51028583938403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>